<commit_message>
Digital press pricing — wire NKK sir's flat Rs/sheet card (2026-06-27)
Sir's hand card: flat Rs/SHEET both-side, up to ~20,000, by paper class x sheet size:
  Art/Maplitho (standard): 12x18=18, 13x19=22 ; Special Paper: 12x18=30, 13x19=35 (4-colour).
- DIGITAL_RATE table + digitalRateFor() + paperIsSpecial(); priceJob now branches on digital:
  printing = Rs/sheet x printed sheets, no plates (replaces the wrong offset-rate borrow).
- isSpecial passed via text + cover params; machine note + breakdown show the digital rate.
- Recorded the card in db/MASTER_DATABASE_2026.xlsx (Digital sheet). Single-colour both-side PENDING.
node-verified digital rates 18/22/30/35; offset path unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/db/MASTER_DATABASE_2026.xlsx
+++ b/db/MASTER_DATABASE_2026.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paper" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Machines (Offset)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Digital press rate" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Press rates (Offset)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Binding" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coating &amp; Embellishment" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hard-case materials rate" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dieline &amp; converting" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wire-O diameters" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="00 README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Paper" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Machines (Offset)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Digital press rate" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Press rates (Offset)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Binding" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Coating &amp; Embellishment" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Hard-case materials rate" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Dieline &amp; converting" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Wire-O diameters" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +79,12 @@
       <b val="1"/>
       <color rgb="0013314F"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0013314F"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -129,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -157,6 +163,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -17562,14 +17578,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
@@ -17785,6 +17801,119 @@
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>PENDING: NKK sir to provide per-click rates per press (and per colour if it varies).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>NKK sir digital rate card (2026-06-27) — FLAT ₹/sheet, printed BOTH SIDES, up to ~20,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Paper class</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Sheet size</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>4-colour both-side ₹/sheet</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Single-colour both-side ₹/sheet</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Art Paper / Maplitho (standard)</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>12 x 18</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>standard = art/maplitho/coated/uncoated</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Art Paper / Maplitho (standard)</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>13 x 19</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="16" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Special Paper</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>12 x 18</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Special Paper</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>13 x 19</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="16" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Single-colour both-side rates PENDING sir. Wired into the app: digital printing = ₹/sheet × printed sheets.</t>
         </is>
       </c>
     </row>

</xml_diff>